<commit_message>
Locklear deck: fix 2 keyword-cannibalization rows in content plan slide
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/locklear-dentistry/keyword-research.xlsx
+++ b/decks/locklear-dentistry/keyword-research.xlsx
@@ -725,7 +725,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -767,7 +766,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -809,7 +807,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -851,7 +848,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -939,7 +935,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -981,7 +976,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1023,7 +1017,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1111,7 +1104,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1153,7 +1145,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1195,7 +1186,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1237,7 +1227,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1279,7 +1268,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1321,7 +1309,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1455,7 +1442,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1497,7 +1483,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1539,7 +1524,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1581,7 +1565,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1623,7 +1606,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1665,7 +1647,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1753,7 +1734,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1795,7 +1775,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1837,7 +1816,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1879,7 +1857,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1899,7 +1876,7 @@
         <v>480</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
@@ -1923,7 +1900,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GSC: 301 impr/90d at pos 31.6. Top emergency money term.</t>
+          <t>GSC: 301 impr/90d at pos 31.6. Top emergency money term. Also targets 'emergency dentist near me' (secondary).</t>
         </is>
       </c>
     </row>
@@ -1933,19 +1910,19 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Need an Emergency Dentist Near You in Greensboro? Start Here</t>
+          <t>Broken or Chipped Tooth in Greensboro? What to Do and Where to Go</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>emergency dentist near me greensboro</t>
+          <t>broken tooth dentist greensboro</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>260</v>
+        <v>110</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
@@ -1969,7 +1946,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>GSC: 'emergency dentist near me' pos 24.6, 107 impr.</t>
+          <t>Retargeted from near-me dup of #31; distinct broken-tooth emergency local page.</t>
         </is>
       </c>
     </row>
@@ -2013,7 +1990,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2055,7 +2031,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2097,7 +2072,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2139,7 +2113,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2181,7 +2154,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2269,7 +2241,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2311,7 +2282,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2353,7 +2323,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2395,7 +2364,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2483,7 +2451,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2525,7 +2492,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2567,7 +2533,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2609,7 +2574,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2697,7 +2661,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2739,7 +2702,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2827,7 +2789,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2869,7 +2830,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2911,7 +2871,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2999,7 +2958,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3041,7 +2999,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3083,7 +3040,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3125,7 +3081,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3213,7 +3168,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3347,7 +3301,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3481,7 +3434,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3523,7 +3475,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3565,7 +3516,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3607,7 +3557,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3649,7 +3598,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3829,7 +3777,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3917,7 +3864,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3959,7 +3905,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -4001,7 +3946,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4043,7 +3987,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4085,7 +4028,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -4127,7 +4069,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -4169,7 +4110,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4211,7 +4151,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4253,7 +4192,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -4295,7 +4233,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4337,7 +4274,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4379,7 +4315,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4421,7 +4356,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4463,7 +4397,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4507,7 +4440,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>GSC: 245-365 impr at pos 28-31. Cosmetic money term.</t>
+          <t>GSC: 245-365 impr at pos 28-31. Cosmetic money term. Also targets 'teeth whitening near me' (secondary).</t>
         </is>
       </c>
     </row>
@@ -4517,19 +4450,19 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Teeth Whitening Near You in Greensboro: What to Know Before You Book</t>
+          <t>How Much Does Teeth Whitening Cost in Greensboro?</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>teeth whitening near me greensboro</t>
+          <t>teeth whitening cost greensboro</t>
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>480</v>
+        <v>90</v>
       </c>
       <c r="E93" s="5" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
@@ -4553,7 +4486,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>GSC: 'teeth whitening near me' pos 23.5, 326 impr.</t>
+          <t>Retargeted from near-me dup of #91; distinct local cost intent.</t>
         </is>
       </c>
     </row>
@@ -4827,7 +4760,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4869,7 +4801,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4911,7 +4842,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -4953,7 +4883,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -4995,7 +4924,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -5037,7 +4965,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -5079,7 +5006,6 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -5121,7 +5047,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -5163,7 +5088,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -5205,7 +5129,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -5247,7 +5170,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -5289,7 +5211,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -5331,7 +5252,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -5373,7 +5293,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -5415,7 +5334,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -5457,7 +5375,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -5499,7 +5416,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -5541,7 +5457,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5583,7 +5498,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5625,7 +5539,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5713,7 +5626,6 @@
           <t>Month 3</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5755,7 +5667,6 @@
           <t>Month 2</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>